<commit_message>
feat(F-NAR-019): ATOM-DIF.PAR.001-06 Le puzzle sous la pluie
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.PAR.001-06.xlsx
+++ b/stories/arbres/ATOM-DIF.PAR.001-06.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>La gare sous la pluie</t>
+          <t>Le puzzle sous la pluie</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>chambre, jour de pluie, tapis beige</t>
+          <t>chambre, jour de pluie, gouttière, zinc, carreau mouillé, ours en tissu, puzzle, tapis beige</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Victorino veut que la locomotive rouge arrive à la gare de bois. Il pleut. Sarah parle peu. Il lui tend un wagon. Ils posent les rails. La locomotive entre en gare.</t>
+          <t>La gouttière chante sur le zinc. Sous la gouttière, un éclat de zinc brille. Victorino veut le puzzle, maintenant. Sarah ne dit rien. Pièce trop vite. Sourire parti, adulte accroupi. Il refuse de foncer, tend, attend. Merci vécu. Pièce du ciel, goutte sur le tapis. Un éclat de zinc tient sous la gouttière.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Les chaussettes épaisses sentent le radiateur. Les gouttes tapent, tapent, tapent. Le carreau est tout mouillé. Une goutte glisse, puis s'arrête. Le zinc fait un petit bruit. Un ours en tissu attend sur l'oreiller. Papa apporte encore une paire. Maman ouvre la caisse des rails. Le bois du tiroir glisse. Les rails sentent le bois neuf. Tu as senti les chaussettes, Victorino ? Elles sont chaudes. On reste au sec, là. Je veux une gare. Pour la locomotive rouge. Une gare sur le tapis ? Oui. Avec un quai. En ce moment, Victorino est sur le tapis. Le tapis est doux et beige. La locomotive rouge attend près de lui. Ses roues sont froides. La porte s'ouvre. Sarah arrive avec son sac. Le sac est mouillé sur le bord. Une goutte tombe sur le tapis. Sarah parle peu. Elle regarde le sol. Victorino a envie de poser beaucoup de questions. Il respire. On peut attendre. Tu peux tendre un jouet. Un wagon bleu est dans sa main. Sarah ne dit rien.</t>
+          <t>La gouttière chante sur le zinc. Ça fait un bruit mince, un peu froid. J'ai entendu le zinc, papa. La gouttière, Victorino ? Oui, papa. Sous la gouttière, un éclat de zinc brille. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Le carreau est mouillé, du bord jusqu'en bas. Une goutte glisse, papa. Sur le carreau ? Oui. Un ours en tissu dort sur l'oreiller. Il a un œil en bouton. Il garde le lit, Victorino ? Oui, maman. Maman ouvre la boîte du puzzle. Le carton sent le papier, un peu. Je veux le puzzle, maintenant ! Les animaux, tout de suite. Le puzzle sur le tapis ? Oui. Avec le chat. En ce moment, Victorino est sur le tapis. Le tapis est beige, un peu rêche. Une pièce du chat attend près de lui. Elle est lisse, papa. Tu la tiens, Victorino ? Oui, papa. La porte s'ouvre. Sarah arrive avec son sac. Le sac est mouillé sur le bord. Tu poses le chat avec moi ? Une goutte tombe sur le tapis. Sarah regarde le sol. Elle ne dit rien. Victorino a envie de tout dire. Le zinc ! L'ours ! Le puzzle ! Victorino pousse trop vite vers elle. La pièce tape la boîte. Oh. Le sourire de Victorino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Sarah, Victorino ? Oui, papa. Tes mains tiennent la pièce, Victorino ? Un peu, maman. L'éclat de zinc tremble, puis tient. Sarah reste près du sac. Elle ne dit rien, papa.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Les chaussettes épaisses sentent le radiateur. Les gouttes tapent, tapent, tapent. Le carreau est tout mouillé. Une goutte glisse, puis s'arrête. Le zinc fait un petit bruit. Un ours en tissu attend sur l'oreiller. Papa apporte encore une paire. Maman ouvre la caisse des rails. Le bois du tiroir glisse. Les rails sentent le bois neuf. Tu as senti les chaussettes, Victorino ? Elles sont chaudes. On reste au sec, là. Je veux une gare. Pour la locomotive rouge. Une gare sur le tapis ? Oui. Avec un quai. En ce moment, Victorino est sur le tapis. Le tapis est doux et beige. La locomotive rouge attend près de lui. Ses roues sont froides. La porte s'ouvre. Sarah arrive avec son sac. Le sac est mouillé sur le bord. Une goutte tombe sur le tapis. Sarah parle peu. Elle regarde le sol. Victorino a envie de poser beaucoup de questions. Il respire. On peut attendre. Tu peux tendre un jouet. Un wagon bleu est dans sa main. Sarah ne dit rien.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La gouttière chante sur le zinc. Ça fait un bruit mince, un peu froid. J'ai entendu le zinc, papa. La gouttière, Victorino ? Oui, papa. Sous la gouttière, un &lt;emphasis level="moderate"&gt;éclat de zinc&lt;/emphasis&gt; brille. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Le carreau est mouillé, du bord jusqu'en bas. Une goutte glisse, papa. Sur le carreau ? Oui. Un ours en tissu dort sur l'oreiller. Il a un œil en bouton. Il garde le lit, Victorino ? Oui, maman. Maman ouvre la boîte du puzzle. Le carton sent le papier, un peu. Je veux le puzzle, maintenant ! Les animaux, tout de suite. Le puzzle sur le tapis ? Oui. Avec le chat. En ce moment, Victorino est sur le tapis. Le tapis est beige, un peu rêche. Une pièce du chat attend près de lui. Elle est lisse, papa. Tu la tiens, Victorino ? Oui, papa. La porte s'ouvre. Sarah arrive avec son sac. Le sac est mouillé sur le bord. Tu poses le chat avec moi ? Une goutte tombe sur le tapis. Sarah regarde le sol. Elle ne dit rien. Victorino a envie de tout dire. Le zinc ! L'ours ! Le puzzle ! Victorino pousse trop vite vers elle. La pièce tape la boîte. Oh. Le sourire de Victorino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Sarah, Victorino ? Oui, papa. Tes mains tiennent la pièce, Victorino ? Un peu, maman. L'éclat de zinc tremble, puis tient. Sarah reste près du sac. Elle ne dit rien, papa.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Aline est dans la chambre. Le tapis est doux. Il pleut dehors. Maman ouvre la porte. Denis arrive avec son sac. Denis parle peu. Il regarde le sol. Aline veut poser beaucoup de questions. Elle ouvre la bouche. Maman dit doucement : on peut &lt;emphasis&gt;attendre&lt;/emphasis&gt;. On n'imite pas. On ne va pas forcer la parole. Aline ferme la bouche. Elle respire. Elle prend un puzzle d'animaux. Elle va tendre un jouet. Elle tend le puzzle vers Denis. Denis regarde. Il ne dit rien. Aline attend. On entend la pluie. Denis prend une pièce. Il la pose. Aline pose une pièce aussi. Papa entre. Il dit : on peut attendre. On peut tendre un jouet. On ne va pas forcer la parole. Denis dit tout bas : le chat. Aline dit : le chat. Ils jouent. Même avec peu de mots. [pause]</t>
+          <t>La gouttière chante sur le zinc. Ça fait un bruit mince, un peu froid. J'ai entendu le zinc, papa. La gouttière, Victorino ? Oui, papa. Sous la gouttière, un &lt;emphasis&gt;éclat de zinc&lt;/emphasis&gt; brille. Il brille, maman. Tu le vois, le petit point ? Oui, un petit point. Le carreau est mouillé, du bord jusqu'en bas. Une goutte glisse, papa. Sur le carreau ? Oui. Un ours en tissu dort sur l'oreiller. Il a un œil en bouton. Il garde le lit, Victorino ? Oui, maman. Maman ouvre la boîte du puzzle. Le carton sent le papier, un peu. Je veux le puzzle, maintenant ! Les animaux, tout de suite. Le puzzle sur le tapis ? Oui. Avec le chat. En ce moment, Victorino est sur le tapis. Le tapis est beige, un peu rêche. Une pièce du chat attend près de lui. Elle est lisse, papa. Tu la tiens, Victorino ? Oui, papa. La porte s'ouvre. Sarah arrive avec son sac. Le sac est mouillé sur le bord. Tu poses le chat avec moi ? Une goutte tombe sur le tapis. Sarah regarde le sol. Elle ne dit rien. Victorino a envie de tout dire. Le zinc ! L'ours ! Le puzzle ! Victorino pousse trop vite vers elle. La pièce tape la boîte. Oh. Le sourire de Victorino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Sarah, Victorino ? Oui, papa. Tes mains tiennent la pièce, Victorino ? Un peu, maman. L'éclat de zinc tremble, puis tient. Sarah reste près du sac. Elle ne dit rien, papa. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>attendre</t>
+          <t>éclat de zinc</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,43 +1326,73 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_le_puzzle_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Les chaussettes épaisses sentent le radiateur.
-narrateur|Les gouttes tapent, tapent, tapent.
-narrateur|Le carreau est tout mouillé.
-narrateur|Une goutte glisse, puis s'arrête.
-narrateur|Le zinc fait un petit bruit.
-narrateur|Un ours en tissu attend sur l'oreiller.
-narrateur|Papa apporte encore une paire.
-narrateur|Maman ouvre la caisse des rails.
-narrateur|Le bois du tiroir glisse.
-narrateur|Les rails sentent le bois neuf.
-papa|Tu as senti les chaussettes, Victorino ?
-enfant-m|Elles sont chaudes.
-maman|On reste au sec, là.
-enfant-m|Je veux une gare.
-enfant-m|Pour la locomotive rouge.
-papa|Une gare sur le tapis ?
+          <t>narrateur|La gouttière chante sur le zinc.
+narrateur|Ça fait un bruit mince, un peu froid.
+enfant-m|J'ai entendu le zinc, papa.
+papa|La gouttière, Victorino ?
+enfant-m|Oui, papa.
+narrateur|Sous la gouttière, un éclat de zinc brille.
+enfant-m|Il brille, maman.
+maman|Tu le vois, le petit point ?
+enfant-m|Oui, un petit point.
+narrateur|Le carreau est mouillé, du bord jusqu'en bas.
+enfant-m|Une goutte glisse, papa.
+papa|Sur le carreau ?
 enfant-m|Oui.
-enfant-m|Avec un quai.
+narrateur|Un ours en tissu dort sur l'oreiller.
+enfant-m|Il a un œil en bouton.
+maman|Il garde le lit, Victorino ?
+enfant-m|Oui, maman.
+narrateur|Maman ouvre la boîte du puzzle.
+narrateur|Le carton sent le papier, un peu.
+enfant-m|Je veux le puzzle, maintenant !
+enfant-m|Les animaux, tout de suite.
+papa|Le puzzle sur le tapis ?
+enfant-m|Oui.
+enfant-m|Avec le chat.
 narrateur|En ce moment, Victorino est sur le tapis.
-narrateur|Le tapis est doux et beige.
-narrateur|La locomotive rouge attend près de lui.
-narrateur|Ses roues sont froides.
+narrateur|Le tapis est beige, un peu rêche.
+narrateur|Une pièce du chat attend près de lui.
+enfant-m|Elle est lisse, papa.
+papa|Tu la tiens, Victorino ?
+enfant-m|Oui, papa.
 narrateur|La porte s'ouvre.
 narrateur|Sarah arrive avec son sac.
 narrateur|Le sac est mouillé sur le bord.
+enfant-m|Tu poses le chat avec moi ?
 narrateur|Une goutte tombe sur le tapis.
-narrateur|Sarah parle peu.
-narrateur|Elle regarde le sol.
-narrateur|Victorino a envie de poser beaucoup de questions.
-narrateur|Il respire.
-maman|On peut attendre.
-papa|Tu peux tendre un jouet.
-narrateur|Un wagon bleu est dans sa main.
-narrateur|Sarah ne dit rien.</t>
+narrateur|Sarah regarde le sol.
+narrateur|Elle ne dit rien.
+narrateur|Victorino a envie de tout dire.
+enfant-m|Le zinc !
+enfant-m|L'ours !
+enfant-m|Le puzzle !
+narrateur|Victorino pousse trop vite vers elle.
+narrateur|La pièce tape la boîte.
+enfant-m|Oh.
+narrateur|Le sourire de Victorino disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Sarah, Victorino ?
+enfant-m|Oui, papa.
+maman|Tes mains tiennent la pièce, Victorino ?
+enfant-m|Un peu, maman.
+narrateur|L'éclat de zinc tremble, puis tient.
+narrateur|Sarah reste près du sac.
+enfant-m|Elle ne dit rien, papa.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>pluie</t>
         </is>
       </c>
     </row>
@@ -1394,12 +1424,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Sarah parle peu. Que fait Victorino ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;&lt;emphasis level="moderate"&gt;Sarah&lt;/emphasis&gt; parle peu. Que fait Victorino ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Denis parle peu. Que fait Aline ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;&lt;emphasis&gt;Sarah&lt;/emphasis&gt; parle peu. Que fait Victorino ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1409,7 +1439,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>attendre | tendre un jouet | un jouet | le wagon | il attend</t>
+          <t>attendre | tendre un jouet | un jouet | elle attend</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1462,7 +1492,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1473,7 +1503,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.22</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1488,34 +1518,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Sarah</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1530,17 +1564,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=sarah_parle_peu_que_fait_victorino; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1573,17 +1607,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Victorino tend le wagon. Pour la gare. Il attend. On entend encore la pluie. Sarah prend le wagon. Elle le pose sur un rail. Clic. On ne force pas la parole. Le train peut rouler sans mots. Victorino pose un autre rail. Le bois fait clic. Sarah pose le quai. Un petit rectangle de bois. La locomotive rouge avance. Elle entre en gare. Les roues s'arrêtent au quai. Elle est arrivée. Puis Sarah dit tout bas. Train. Train. Tu as su attendre. Bravo, Victorino. L'ours regarde depuis l'oreiller. Un œil en bouton brille. La locomotive reste au quai.</t>
+          <t>Victorino veut le puzzle, tout de suite. Je la pose, maintenant ! Il avance trop vite vers Sarah. Les mots se bousculent dans sa bouche. Sarah baisse les yeux. Elle serre le sac contre elle. Oh. Le sourire ne revient pas. Victorino refuse de foncer. Il referme la bouche. Personne ne parle. Il observe la pièce, un instant. Il écoute la gouttière sur le zinc. Tu veux le puzzle avec Sarah ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose la pièce, puis on reste. D'accord. Victorino reste un moment, les mains ouvertes. Il attend. Il tend la pièce du chat. Pour toi. Sarah ne dit rien. Elle prend la pièce, sans parler. Oui. Victorino pose les mains sur le tapis. Il reste, sans se presser. Sarah pose le chat, plus lentement. Merci, Victorino. Papa a vu les deux, dans la chambre. Le carton est tiède, sous les doigts. Il est chaud. Le chat tient, un peu de travers. Le chat. Il a une oreille, là ? Oui, là. Victorino glisse le doigt sur le carton. Le papier est doux, contre la peau. Tes mains sont au chaud, Victorino ? Un peu, maman. Sarah s'assoit, puis se relève. Chat. On va jusqu'au bord ? Le tapis beige va jusqu'au mur. Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Victorino tend le wagon. Pour la gare. Il attend. On entend encore la pluie. Sarah prend le wagon. Elle le pose sur un rail. Clic. On ne force pas la parole. Le train peut rouler sans mots. Victorino pose un autre rail. Le bois fait clic. Sarah pose le quai. Un petit rectangle de bois. La locomotive rouge avance. Elle entre en gare. Les roues s'arrêtent au quai. Elle est arrivée. Puis Sarah dit tout bas. Train. Train. Tu as su attendre. Bravo, Victorino. L'ours regarde depuis l'oreiller. Un œil en bouton brille. La locomotive reste au quai.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorino veut le &lt;emphasis level="moderate"&gt;puzzle&lt;/emphasis&gt;, tout de suite. Je la pose, maintenant ! Il avance trop vite vers Sarah. Les mots se bousculent dans sa bouche. Sarah baisse les yeux. Elle serre le sac contre elle. Oh. Le sourire ne revient pas. Victorino refuse de foncer. Il referme la bouche. Personne ne parle. Il observe la pièce, un instant. Il écoute la gouttière sur le zinc. Tu veux le puzzle avec Sarah ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose la pièce, puis on reste. D'accord. Victorino reste un moment, les mains ouvertes. Il attend. Il tend la pièce du chat. Pour toi. Sarah ne dit rien. Elle prend la pièce, sans parler. Oui. Victorino pose les mains sur le tapis. Il reste, sans se presser. Sarah pose le chat, plus lentement. Merci, Victorino. Papa a vu les deux, dans la chambre. Le carton est tiède, sous les doigts. Il est chaud. Le chat tient, un peu de travers. Le chat. Il a une oreille, là ? Oui, là. Victorino glisse le doigt sur le carton. Le papier est doux, contre la peau. Tes mains sont au chaud, Victorino ? Un peu, maman. Sarah s'assoit, puis se relève. Chat. On va jusqu'au bord ? Le tapis beige va jusqu'au mur. Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Aline a su &lt;emphasis&gt;attendre&lt;/emphasis&gt;. Elle a tendu un jouet. Denis a pris une pièce. On n'a pas forcé la parole. [pause]</t>
+          <t>Victorino veut le &lt;emphasis&gt;puzzle&lt;/emphasis&gt;, tout de suite. Je la pose, maintenant ! Il avance trop vite vers Sarah. Les mots se bousculent dans sa bouche. Sarah baisse les yeux. Elle serre le sac contre elle. Oh. Le sourire ne revient pas. Victorino refuse de foncer. Il referme la bouche. Personne ne parle. Il observe la pièce, un instant. Il écoute la gouttière sur le zinc. Tu veux le puzzle avec Sarah ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose la pièce, puis on reste. D'accord. Victorino reste un moment, les mains ouvertes. Il attend. Il tend la pièce du chat. Pour toi. Sarah ne dit rien. Elle prend la pièce, sans parler. Oui. Victorino pose les mains sur le tapis. Il reste, sans se presser. Sarah pose le chat, plus lentement. Merci, Victorino. Papa a vu les deux, dans la chambre. Le carton est tiède, sous les doigts. Il est chaud. Le chat tient, un peu de travers. Le chat. Il a une oreille, là ? Oui, là. Victorino glisse le doigt sur le carton. Le papier est doux, contre la peau. Tes mains sont au chaud, Victorino ? Un peu, maman. Sarah s'assoit, puis se relève. Chat. On va jusqu'au bord ? Le tapis beige va jusqu'au mur. Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1630,7 +1664,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1638,10 +1672,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1664,30 +1698,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>attendre</t>
+          <t>puzzle</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1696,10 +1730,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1712,36 +1746,61 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_attend_tend; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Victorino tend le wagon.
-enfant-m|Pour la gare.
+          <t>narrateur|Victorino veut le puzzle, tout de suite.
+enfant-m|Je la pose, maintenant !
+narrateur|Il avance trop vite vers Sarah.
+narrateur|Les mots se bousculent dans sa bouche.
+narrateur|Sarah baisse les yeux.
+narrateur|Elle serre le sac contre elle.
+enfant-m|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Victorino refuse de foncer.
+narrateur|Il referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Il observe la pièce, un instant.
+narrateur|Il écoute la gouttière sur le zinc.
+papa|Tu veux le puzzle avec Sarah ?
+narrateur|Papa reste à la même hauteur.
+enfant-m|Papa, on fait quoi ?
+papa|On pose la pièce, puis on reste.
+enfant-m|D'accord.
+narrateur|Victorino reste un moment, les mains ouvertes.
 narrateur|Il attend.
-narrateur|On entend encore la pluie.
-narrateur|Sarah prend le wagon.
-narrateur|Elle le pose sur un rail.
-narrateur|Clic.
-maman|On ne force pas la parole.
-papa|Le train peut rouler sans mots.
-narrateur|Victorino pose un autre rail.
-narrateur|Le bois fait clic.
-narrateur|Sarah pose le quai.
-narrateur|Un petit rectangle de bois.
-narrateur|La locomotive rouge avance.
-narrateur|Elle entre en gare.
-narrateur|Les roues s'arrêtent au quai.
-enfant-m|Elle est arrivée.
-narrateur|Puis Sarah dit tout bas.
-enfant-f|Train.
-enfant-m|Train.
-papa|Tu as su attendre.
-papa|Bravo, Victorino.
-narrateur|L'ours regarde depuis l'oreiller.
-narrateur|Un œil en bouton brille.
-narrateur|La locomotive reste au quai.</t>
+narrateur|Il tend la pièce du chat.
+enfant-m|Pour toi.
+narrateur|Sarah ne dit rien.
+narrateur|Elle prend la pièce, sans parler.
+copine|Oui.
+narrateur|Victorino pose les mains sur le tapis.
+narrateur|Il reste, sans se presser.
+narrateur|Sarah pose le chat, plus lentement.
+papa|Merci, Victorino.
+narrateur|Papa a vu les deux, dans la chambre.
+maman|Le carton est tiède, sous les doigts.
+enfant-m|Il est chaud.
+narrateur|Le chat tient, un peu de travers.
+enfant-m|Le chat.
+papa|Il a une oreille, là ?
+enfant-m|Oui, là.
+narrateur|Victorino glisse le doigt sur le carton.
+narrateur|Le papier est doux, contre la peau.
+maman|Tes mains sont au chaud, Victorino ?
+enfant-m|Un peu, maman.
+narrateur|Sarah s'assoit, puis se relève.
+copine|Chat.
+enfant-m|On va jusqu'au bord ?
+maman|Le tapis beige va jusqu'au mur.
+enfant-m|Oui, maman.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>pluie</t>
         </is>
       </c>
     </row>
@@ -1768,17 +1827,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Maman apporte deux bols. La soupe sent la carotte. Un peu de soupe ? Sarah secoue la tête. D'accord. D'accord. Tu as fini la gare, Victorino ? Oui, maman. La locomotive est au quai. Maman aide Sarah à mettre son manteau. Le manteau est encore un peu humide. Sarah fait un petit signe. À demain ? À demain. Les chaussettes sèchent encore. L'ours attend sur l'oreiller. La pluie chante encore un peu. Le zinc aussi. Oui. Il chante encore.</t>
+          <t>Ils restent sur le tapis beige. Une pièce du ciel manque, au milieu. Je la mets, maintenant ! Victorino pousse trop vite. La pièce glisse vers la goutte. Ça tombe ! Sarah tend les mains, sans parler. Victorino avance les mains, trop vite. Puis il s'arrête net. Victorino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe la pièce, un instant. Il écoute la gouttière, sur le zinc. Près du carreau, un éclat de zinc luit. Là, sur le zinc. Tu prends le ciel, Sarah ? Sarah ne dit rien. Elle tend les mains, sans parler. Oui. Victorino passe la pièce, sans se presser. Sarah la pose, plus lentement. Le carton est lisse et un peu froid. Tu le vois, le ciel ? Oui, papa. Le tapis beige est près du mur ? Oui, maman. La pièce entre dans le trou. Victorino pose une main sur le carton. Sarah pose la suivante. Le puzzle tient, Victorino ? Oui, papa. Une goutte passe sur le carreau. Elle allume le zinc.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Maman apporte deux bols. La soupe sent la carotte. Un peu de soupe ? Sarah secoue la tête. D'accord. D'accord. Tu as fini la gare, Victorino ? Oui, maman. La locomotive est au quai. Maman aide Sarah à mettre son manteau. Le manteau est encore un peu humide. Sarah fait un petit signe. À demain ? À demain. Les chaussettes sèchent encore. L'ours attend sur l'oreiller. La pluie chante encore un peu. Le zinc aussi. Oui. Il chante encore.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils restent sur le tapis beige. Une pièce du ciel manque, au milieu. Je la mets, maintenant ! Victorino pousse trop vite. La pièce glisse vers la goutte. Ça tombe ! Sarah tend les mains, sans parler. Victorino avance les mains, trop vite. Puis il s'arrête net. Victorino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe la pièce, un instant. Il écoute la gouttière, sur le zinc. Près du carreau, un &lt;emphasis level="moderate"&gt;éclat de zinc&lt;/emphasis&gt; luit. Là, sur le zinc. Tu prends le ciel, Sarah ? Sarah ne dit rien. Elle tend les mains, sans parler. Oui. Victorino passe la pièce, sans se presser. Sarah la pose, plus lentement. Le carton est lisse et un peu froid. Tu le vois, le ciel ? Oui, papa. Le tapis beige est près du mur ? Oui, maman. La pièce entre dans le trou. Victorino pose une main sur le carton. Sarah pose la suivante. Le puzzle tient, Victorino ? Oui, papa. Une goutte passe sur le carreau. Elle allume le zinc.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman aide Denis à mettre son manteau. Denis fait un petit signe. Aline range le puzzle. [pause]</t>
+          <t>Ils restent sur le tapis beige. Une pièce du ciel manque, au milieu. Je la mets, maintenant ! Victorino pousse trop vite. La pièce glisse vers la goutte. Ça tombe ! Sarah tend les mains, sans parler. Victorino avance les mains, trop vite. Puis il s'arrête net. Victorino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe la pièce, un instant. Il écoute la gouttière, sur le zinc. Près du carreau, un &lt;emphasis&gt;éclat de zinc&lt;/emphasis&gt; luit. Là, sur le zinc. Tu prends le ciel, Sarah ? Sarah ne dit rien. Elle tend les mains, sans parler. Oui. Victorino passe la pièce, sans se presser. Sarah la pose, plus lentement. Le carton est lisse et un peu froid. Tu le vois, le ciel ? Oui, papa. Le tapis beige est près du mur ? Oui, maman. La pièce entre dans le trou. Victorino pose une main sur le carton. Sarah pose la suivante. Le puzzle tient, Victorino ? Oui, papa. Une goutte passe sur le carreau. Elle allume le zinc. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1825,7 +1884,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1833,10 +1892,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1857,28 +1916,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de zinc</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1887,10 +1950,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1901,29 +1964,52 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=piece_du_ciel_goutte_il_s_arrete; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Maman apporte deux bols.
-narrateur|La soupe sent la carotte.
-maman|Un peu de soupe ?
-narrateur|Sarah secoue la tête.
-enfant-m|D'accord.
-papa|D'accord.
-maman|Tu as fini la gare, Victorino ?
+          <t>narrateur|Ils restent sur le tapis beige.
+narrateur|Une pièce du ciel manque, au milieu.
+enfant-m|Je la mets, maintenant !
+narrateur|Victorino pousse trop vite.
+narrateur|La pièce glisse vers la goutte.
+enfant-m|Ça tombe !
+narrateur|Sarah tend les mains, sans parler.
+narrateur|Victorino avance les mains, trop vite.
+narrateur|Puis il s'arrête net.
+narrateur|Victorino refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Il observe la pièce, un instant.
+narrateur|Il écoute la gouttière, sur le zinc.
+narrateur|Près du carreau, un éclat de zinc luit.
+enfant-m|Là, sur le zinc.
+enfant-m|Tu prends le ciel, Sarah ?
+narrateur|Sarah ne dit rien.
+narrateur|Elle tend les mains, sans parler.
+copine|Oui.
+narrateur|Victorino passe la pièce, sans se presser.
+narrateur|Sarah la pose, plus lentement.
+narrateur|Le carton est lisse et un peu froid.
+papa|Tu le vois, le ciel ?
+enfant-m|Oui, papa.
+maman|Le tapis beige est près du mur ?
 enfant-m|Oui, maman.
-enfant-m|La locomotive est au quai.
-narrateur|Maman aide Sarah à mettre son manteau.
-narrateur|Le manteau est encore un peu humide.
-narrateur|Sarah fait un petit signe.
-papa|À demain ?
-enfant-m|À demain.
-narrateur|Les chaussettes sèchent encore.
-narrateur|L'ours attend sur l'oreiller.
-narrateur|La pluie chante encore un peu.
-enfant-m|Le zinc aussi.
-papa|Oui.
-papa|Il chante encore.</t>
+narrateur|La pièce entre dans le trou.
+narrateur|Victorino pose une main sur le carton.
+narrateur|Sarah pose la suivante.
+papa|Le puzzle tient, Victorino ?
+enfant-m|Oui, papa.
+maman|Une goutte passe sur le carreau.
+enfant-m|Elle allume le zinc.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>pluie</t>
         </is>
       </c>
     </row>
@@ -1950,17 +2036,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le train est en gare. Même sous la pluie. Le quai est prêt.</t>
+          <t>Ils restent près du tapis. Le puzzle est arrivé, Victorino ? Oui, maman. Tu souffles un peu ? Oui, papa. Victorino souffle, un filet d'air. Le carton sent le papier. Tu le sens, le puzzle ? Oui, maman. Le chat reste un peu, de travers. Il a tenu, sur le tapis. Chat. Le tapis est tiède, sous les mains. L'ours regarde depuis l'oreiller. On y retourne, après. Un éclat de zinc tient sous la gouttière.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le train est en gare. Même sous la pluie. Le quai est prêt.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près du tapis. Le puzzle est arrivé, Victorino ? Oui, maman. Tu souffles un peu ? Oui, papa. Victorino souffle, un filet d'air. Le carton sent le papier. Tu le sens, le puzzle ? Oui, maman. Le chat reste un peu, de travers. Il a tenu, sur le tapis. Chat. Le tapis est tiède, sous les mains. L'ours regarde depuis l'oreiller. On y retourne, après. Un &lt;emphasis level="moderate"&gt;éclat de zinc&lt;/emphasis&gt; tient sous la gouttière.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près du tapis. Le puzzle est arrivé, Victorino ? Oui, maman. Tu souffles un peu ? Oui, papa. Victorino souffle, un filet d'air. Le carton sent le papier. Tu le sens, le puzzle ? Oui, maman. Le chat reste un peu, de travers. Il a tenu, sur le tapis. Chat. Le tapis est tiède, sous les mains. L'ours regarde depuis l'oreiller. On y retourne, après. Un &lt;emphasis&gt;éclat de zinc&lt;/emphasis&gt; tient sous la gouttière.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2007,15 +2093,15 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.28</v>
@@ -2027,12 +2113,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2041,17 +2127,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de zinc</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2060,11 +2150,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2073,26 +2163,43 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sous_la_gouttiere; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|Le train est en gare.
-maman|Même sous la pluie.
-papa|Le quai est prêt.</t>
+          <t>narrateur|Ils restent près du tapis.
+maman|Le puzzle est arrivé, Victorino ?
+enfant-m|Oui, maman.
+papa|Tu souffles un peu ?
+enfant-m|Oui, papa.
+narrateur|Victorino souffle, un filet d'air.
+enfant-m|Le carton sent le papier.
+maman|Tu le sens, le puzzle ?
+enfant-m|Oui, maman.
+papa|Le chat reste un peu, de travers.
+enfant-m|Il a tenu, sur le tapis.
+copine|Chat.
+narrateur|Le tapis est tiède, sous les mains.
+narrateur|L'ours regarde depuis l'oreiller.
+enfant-m|On y retourne, après.
+narrateur|Un éclat de zinc tient sous la gouttière.</t>
         </is>
       </c>
     </row>
@@ -2113,7 +2220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2170,6 +2277,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>